<commit_message>
sube el latex al repo
</commit_message>
<xml_diff>
--- a/hardware/Circuito Final/Circuito externo/Pines controlador.xlsx
+++ b/hardware/Circuito Final/Circuito externo/Pines controlador.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\---\Desktop\Tesis\hardware\Circuito Final\Circuito externo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B2C900-9C18-4EF0-8B18-3F995D7ED9C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="105">
   <si>
     <t>PC10</t>
   </si>
@@ -58,9 +57,6 @@
     <t>PB9</t>
   </si>
   <si>
-    <t>ADC15</t>
-  </si>
-  <si>
     <t>PC5</t>
   </si>
   <si>
@@ -87,6 +83,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PA5</t>
     </r>
@@ -96,6 +93,7 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>/</t>
     </r>
@@ -104,14 +102,12 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PB13</t>
     </r>
   </si>
   <si>
-    <t>ADC5</t>
-  </si>
-  <si>
     <t>PA12</t>
   </si>
   <si>
@@ -126,6 +122,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PA6</t>
     </r>
@@ -135,6 +132,7 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>/</t>
     </r>
@@ -143,14 +141,12 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PB14</t>
     </r>
   </si>
   <si>
-    <t>ADC6</t>
-  </si>
-  <si>
     <t>PA11</t>
   </si>
   <si>
@@ -162,6 +158,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PA7</t>
     </r>
@@ -171,6 +168,7 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>/</t>
     </r>
@@ -179,14 +177,12 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PB15</t>
     </r>
   </si>
   <si>
-    <t>ADC7</t>
-  </si>
-  <si>
     <t>PB12</t>
   </si>
   <si>
@@ -240,6 +236,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PB15</t>
     </r>
@@ -248,6 +245,7 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>/PA7</t>
     </r>
@@ -256,9 +254,6 @@
     <t>PC15</t>
   </si>
   <si>
-    <t>ADC0</t>
-  </si>
-  <si>
     <t>PA0</t>
   </si>
   <si>
@@ -270,6 +265,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PB14</t>
     </r>
@@ -278,6 +274,7 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>/PA6</t>
     </r>
@@ -286,9 +283,6 @@
     <t>PD0</t>
   </si>
   <si>
-    <t>ADC1</t>
-  </si>
-  <si>
     <t>PA1</t>
   </si>
   <si>
@@ -300,6 +294,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PB13</t>
     </r>
@@ -308,6 +303,7 @@
         <sz val="10"/>
         <color rgb="FFCCCCCC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>/PA5</t>
     </r>
@@ -334,18 +330,12 @@
     <t>PA10</t>
   </si>
   <si>
-    <t>ADC14</t>
-  </si>
-  <si>
     <t>PC4</t>
   </si>
   <si>
     <t>PC2</t>
   </si>
   <si>
-    <t>ADC12</t>
-  </si>
-  <si>
     <t>ADC11</t>
   </si>
   <si>
@@ -354,6 +344,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PC1</t>
     </r>
@@ -362,6 +353,7 @@
         <sz val="10"/>
         <color rgb="FFD9D9D9"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>/PB9</t>
     </r>
@@ -373,17 +365,12 @@
     <t>PC3</t>
   </si>
   <si>
-    <t>ADC13</t>
-  </si>
-  <si>
-    <t>ADC10</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PC0</t>
     </r>
@@ -392,6 +379,7 @@
         <sz val="10"/>
         <color rgb="FFD9D9D9"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>/PB8</t>
     </r>
@@ -476,12 +464,48 @@
   </si>
   <si>
     <t>bus_neg4</t>
+  </si>
+  <si>
+    <t>vcc stm</t>
+  </si>
+  <si>
+    <t>salida_adc_1</t>
+  </si>
+  <si>
+    <t>banco1_med</t>
+  </si>
+  <si>
+    <t>medicion_corriente_de_carga</t>
+  </si>
+  <si>
+    <t>salida_adc_2</t>
+  </si>
+  <si>
+    <t>banco2_med</t>
+  </si>
+  <si>
+    <t>salida_adc_3</t>
+  </si>
+  <si>
+    <t>salida_adc_4</t>
+  </si>
+  <si>
+    <t>banco4_med</t>
+  </si>
+  <si>
+    <t>medicion_corriente_descarga</t>
+  </si>
+  <si>
+    <t>banco3_med</t>
+  </si>
+  <si>
+    <t>llave de emergencia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -493,34 +517,40 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFD9D2E9"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFCCCCCC"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFCCCCCC"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFD9D9D9"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -549,7 +579,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -596,6 +626,12 @@
       <patternFill patternType="solid">
         <fgColor theme="6"/>
         <bgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -701,7 +737,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -772,6 +808,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -991,12 +1033,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="B1:T35"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="7" width="13.85546875" customWidth="1"/>
   </cols>
@@ -1012,10 +1054,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>1</v>
@@ -1030,10 +1072,10 @@
         <v>2</v>
       </c>
       <c r="K2" s="23" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="L2" s="24" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>3</v>
@@ -1042,13 +1084,13 @@
         <v>1</v>
       </c>
       <c r="P2" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="S2" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="S2" s="21" t="s">
-        <v>87</v>
-      </c>
       <c r="T2" s="21" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1074,7 +1116,7 @@
       </c>
       <c r="K3" s="12"/>
       <c r="L3" s="25" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>8</v>
@@ -1083,13 +1125,13 @@
         <v>3</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="S3" s="21" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="T3" s="21" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1115,22 +1157,22 @@
       </c>
       <c r="K4" s="12"/>
       <c r="L4" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N4" s="26">
+      <c r="N4" s="30">
         <v>5</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="S4" s="21" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="T4" s="21" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1138,12 +1180,12 @@
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="14"/>
       <c r="F5" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G5" s="26">
         <v>7</v>
@@ -1152,24 +1194,24 @@
         <v>8</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K5" s="12"/>
       <c r="L5" s="14"/>
       <c r="M5" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N5" s="26">
         <v>7</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="S5" s="21" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="T5" s="21" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1177,12 +1219,12 @@
         <v>10</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" s="12"/>
       <c r="E6" s="14"/>
       <c r="F6" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G6" s="26">
         <v>9</v>
@@ -1191,24 +1233,24 @@
         <v>10</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K6" s="12"/>
       <c r="L6" s="14"/>
       <c r="M6" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N6" s="26">
         <v>9</v>
       </c>
       <c r="P6" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="S6" s="21" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="T6" s="21" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1216,42 +1258,42 @@
         <v>12</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7" s="12"/>
       <c r="E7" s="14"/>
       <c r="F7" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G7" s="26">
         <v>11</v>
       </c>
-      <c r="I7" s="27">
+      <c r="I7" s="29">
         <v>12</v>
       </c>
       <c r="J7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="L7" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="M7" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="L7" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="N7" s="26">
         <v>11</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="S7" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="T7" s="21" t="s">
         <v>86</v>
-      </c>
-      <c r="T7" s="21" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="8" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1259,14 +1301,14 @@
         <v>14</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D8" s="28" t="s">
         <v>5</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G8" s="26">
         <v>13</v>
@@ -1275,16 +1317,16 @@
         <v>14</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>26</v>
+        <v>102</v>
       </c>
       <c r="L8" s="25" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N8" s="26">
         <v>13</v>
@@ -1293,7 +1335,7 @@
         <v>5</v>
       </c>
       <c r="T8" s="21" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1301,37 +1343,39 @@
         <v>16</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D9" s="16"/>
-      <c r="E9" s="14"/>
+      <c r="E9" s="14" t="s">
+        <v>93</v>
+      </c>
       <c r="F9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G9" s="26">
         <v>15</v>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="29">
         <v>16</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="L9" s="14"/>
       <c r="M9" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="N9" s="26">
         <v>15</v>
       </c>
       <c r="S9" s="21" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="T9" s="21" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1339,12 +1383,12 @@
         <v>18</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="14"/>
       <c r="F10" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G10" s="26">
         <v>17</v>
@@ -1353,21 +1397,21 @@
         <v>18</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="K10" s="12"/>
       <c r="L10" s="14"/>
       <c r="M10" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N10" s="26">
         <v>17</v>
       </c>
       <c r="S10" s="21" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="T10" s="21" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1375,12 +1419,12 @@
         <v>20</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="14"/>
       <c r="F11" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G11" s="26">
         <v>19</v>
@@ -1389,21 +1433,21 @@
         <v>20</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="K11" s="16"/>
       <c r="L11" s="14"/>
       <c r="M11" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N11" s="26">
         <v>19</v>
       </c>
       <c r="S11" s="21" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="T11" s="21" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1411,12 +1455,12 @@
         <v>22</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="14"/>
       <c r="F12" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G12" s="26">
         <v>21</v>
@@ -1425,18 +1469,18 @@
         <v>22</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="K12" s="16"/>
       <c r="L12" s="14"/>
       <c r="M12" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="N12" s="26">
         <v>21</v>
       </c>
       <c r="T12" s="21" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1444,14 +1488,14 @@
         <v>24</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E13" s="14"/>
       <c r="F13" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G13" s="26">
         <v>23</v>
@@ -1460,18 +1504,18 @@
         <v>24</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="K13" s="16"/>
       <c r="L13" s="14"/>
       <c r="M13" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="N13" s="26">
         <v>23</v>
       </c>
       <c r="T13" s="21" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1479,12 +1523,12 @@
         <v>26</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="14"/>
       <c r="F14" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G14" s="26">
         <v>25</v>
@@ -1493,18 +1537,18 @@
         <v>26</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="K14" s="12"/>
       <c r="L14" s="14"/>
       <c r="M14" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="N14" s="26">
         <v>25</v>
       </c>
       <c r="T14" s="21" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1512,28 +1556,28 @@
         <v>28</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="13" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G15" s="26">
+        <v>45</v>
+      </c>
+      <c r="G15" s="30">
         <v>27</v>
       </c>
       <c r="I15" s="27">
         <v>28</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="K15" s="12"/>
       <c r="L15" s="14"/>
       <c r="M15" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="N15" s="26">
         <v>27</v>
@@ -1544,28 +1588,28 @@
         <v>30</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="13" t="s">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G16" s="26">
+        <v>49</v>
+      </c>
+      <c r="G16" s="30">
         <v>29</v>
       </c>
       <c r="I16" s="27">
         <v>30</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="K16" s="12"/>
       <c r="L16" s="14"/>
       <c r="M16" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="N16" s="26">
         <v>29</v>
@@ -1576,14 +1620,14 @@
         <v>32</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="G17" s="26">
         <v>31</v>
@@ -1592,12 +1636,12 @@
         <v>32</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="K17" s="12"/>
       <c r="L17" s="14"/>
       <c r="M17" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="N17" s="26">
         <v>31</v>
@@ -1613,7 +1657,7 @@
       <c r="D18" s="12"/>
       <c r="E18" s="22"/>
       <c r="F18" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="G18" s="26">
         <v>33</v>
@@ -1622,34 +1666,36 @@
         <v>34</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="K18" s="16"/>
+        <v>58</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>104</v>
+      </c>
       <c r="L18" s="13" t="s">
-        <v>65</v>
+        <v>99</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="N18" s="26">
+        <v>59</v>
+      </c>
+      <c r="N18" s="30">
         <v>33</v>
       </c>
     </row>
     <row r="19" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="27">
+      <c r="B19" s="29">
         <v>36</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="G19" s="26">
         <v>35</v>
@@ -1658,32 +1704,32 @@
         <v>36</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="K19" s="12"/>
       <c r="L19" s="14"/>
       <c r="M19" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N19" s="26">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="2:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="27">
+      <c r="B20" s="29">
         <v>38</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G20" s="26">
         <v>37</v>
@@ -1692,12 +1738,12 @@
         <v>38</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="K20" s="17"/>
       <c r="L20" s="18"/>
       <c r="M20" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N20" s="26">
         <v>37</v>

</xml_diff>